<commit_message>
test/update landing execution test cases.
</commit_message>
<xml_diff>
--- a/TestCases_Docs/Landing_TestCases.xlsx
+++ b/TestCases_Docs/Landing_TestCases.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenovo\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\iti\QA\New folder\Clothing-Web-Portal\TestCases_Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D50CE504-973C-4049-A768-D5F0239DA92D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22CB61AC-407D-4B79-BE59-43E1CFA6A257}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Landing Test Cases" sheetId="5" r:id="rId1"/>
@@ -1225,9 +1225,6 @@
     <t>Execution_Status</t>
   </si>
   <si>
-    <t>Failed</t>
-  </si>
-  <si>
     <t>TC_Landing_001</t>
   </si>
   <si>
@@ -1340,6 +1337,9 @@
   </si>
   <si>
     <t>redirected to /customer/orders</t>
+  </si>
+  <si>
+    <t>Passed</t>
   </si>
 </sst>
 </file>
@@ -1807,59 +1807,6 @@
   </cellStyles>
   <dxfs count="60">
     <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill>
           <bgColor theme="7"/>
@@ -1874,29 +1821,6 @@
       </fill>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
       <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
@@ -2050,6 +1974,25 @@
       </border>
     </dxf>
     <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
       <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
@@ -2064,6 +2007,23 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -2316,6 +2276,29 @@
       </border>
     </dxf>
     <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
       <font>
         <color theme="1"/>
         <family val="2"/>
@@ -2334,6 +2317,23 @@
         <bottom style="thin">
           <color rgb="FF000000"/>
         </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
         <vertical/>
         <horizontal/>
       </border>
@@ -2677,42 +2677,42 @@
     <tableColumn id="3" xr3:uid="{7853AC75-B7A3-4B9B-B597-0CC90E8D52BF}" name="valid/invalid" dataDxfId="36"/>
     <tableColumn id="4" xr3:uid="{AAABAF80-25C1-4ACB-ADF4-7337AEA0E0A4}" name="Environment" dataDxfId="35"/>
     <tableColumn id="5" xr3:uid="{050A3DD3-5C3B-40E3-B68A-DE6E46C20CD3}" name="Pre-condition" dataDxfId="34"/>
-    <tableColumn id="6" xr3:uid="{695FB61F-899E-47FB-AC04-D25E8F4EFFA9}" name="Steps" dataDxfId="0"/>
-    <tableColumn id="7" xr3:uid="{6AADAA49-15BA-4E3C-B63A-DDA3E7EF4C96}" name="Test Data" dataDxfId="33"/>
-    <tableColumn id="8" xr3:uid="{C1CE8F53-60B8-411D-A252-48EAF0B6899D}" name="Expected Results" dataDxfId="5"/>
-    <tableColumn id="9" xr3:uid="{5CBA8F0E-EFB2-441E-ABB2-C8AFC9733678}" name="Post Condition" dataDxfId="32"/>
-    <tableColumn id="10" xr3:uid="{F1F2F7F1-026F-45A0-971C-F5B647193AEB}" name="TC Status" dataDxfId="31"/>
-    <tableColumn id="11" xr3:uid="{C1B2E8E9-0DE1-4E62-B972-DE5006C951AE}" name="Attachment" dataDxfId="30"/>
-    <tableColumn id="12" xr3:uid="{3F1A62C0-FBFC-41F2-B1C9-42BCC073A738}" name="Requirement ID" dataDxfId="29"/>
-    <tableColumn id="13" xr3:uid="{FF0D4754-9DCA-4527-96A7-45E4EA4C6EED}" name="Type" dataDxfId="28"/>
-    <tableColumn id="14" xr3:uid="{CEE95E6B-C591-4C14-8305-FA320F301C59}" name="Tester" dataDxfId="27"/>
-    <tableColumn id="15" xr3:uid="{678D806D-10AD-4D08-AE9F-776FEBFD7C5C}" name="Comment" dataDxfId="26"/>
+    <tableColumn id="6" xr3:uid="{695FB61F-899E-47FB-AC04-D25E8F4EFFA9}" name="Steps" dataDxfId="33"/>
+    <tableColumn id="7" xr3:uid="{6AADAA49-15BA-4E3C-B63A-DDA3E7EF4C96}" name="Test Data" dataDxfId="32"/>
+    <tableColumn id="8" xr3:uid="{C1CE8F53-60B8-411D-A252-48EAF0B6899D}" name="Expected Results" dataDxfId="31"/>
+    <tableColumn id="9" xr3:uid="{5CBA8F0E-EFB2-441E-ABB2-C8AFC9733678}" name="Post Condition" dataDxfId="30"/>
+    <tableColumn id="10" xr3:uid="{F1F2F7F1-026F-45A0-971C-F5B647193AEB}" name="TC Status" dataDxfId="29"/>
+    <tableColumn id="11" xr3:uid="{C1B2E8E9-0DE1-4E62-B972-DE5006C951AE}" name="Attachment" dataDxfId="28"/>
+    <tableColumn id="12" xr3:uid="{3F1A62C0-FBFC-41F2-B1C9-42BCC073A738}" name="Requirement ID" dataDxfId="27"/>
+    <tableColumn id="13" xr3:uid="{FF0D4754-9DCA-4527-96A7-45E4EA4C6EED}" name="Type" dataDxfId="26"/>
+    <tableColumn id="14" xr3:uid="{CEE95E6B-C591-4C14-8305-FA320F301C59}" name="Tester" dataDxfId="25"/>
+    <tableColumn id="15" xr3:uid="{678D806D-10AD-4D08-AE9F-776FEBFD7C5C}" name="Comment" dataDxfId="24"/>
   </tableColumns>
   <tableStyleInfo name="Cart Test Cases-style" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{7DE26239-599D-4E8A-B29E-9F20DE12A166}" name="Table1719" displayName="Table1719" ref="A1:Q8" totalsRowShown="0" headerRowDxfId="25" dataDxfId="23" headerRowBorderDxfId="24" tableBorderDxfId="22" totalsRowBorderDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{7DE26239-599D-4E8A-B29E-9F20DE12A166}" name="Table1719" displayName="Table1719" ref="A1:Q8" totalsRowShown="0" headerRowDxfId="23" dataDxfId="21" headerRowBorderDxfId="22" tableBorderDxfId="20" totalsRowBorderDxfId="19">
   <autoFilter ref="A1:Q8" xr:uid="{CA9B46E1-5155-4AAF-844B-BCD9CCA2EDF6}"/>
   <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{6349AC1B-18C1-4513-A98D-74004451BE07}" name="TesTCASE ID" dataDxfId="20"/>
-    <tableColumn id="2" xr3:uid="{316A01E1-D06A-4667-AE3C-453DBC4B1054}" name="Test Cases Title " dataDxfId="19"/>
-    <tableColumn id="3" xr3:uid="{8F7A3C5E-7DAA-4BE5-BB4C-4242660A0347}" name="valid/invalid" dataDxfId="18"/>
-    <tableColumn id="4" xr3:uid="{6F77ADFD-1C3F-4A08-A6E4-478BE3CD7F59}" name="Environment" dataDxfId="17"/>
-    <tableColumn id="5" xr3:uid="{519F839C-1B74-4449-9BE1-EDCA27C25137}" name="Pre-condition" dataDxfId="16"/>
-    <tableColumn id="6" xr3:uid="{F29F0414-7871-4D01-A1DD-A280EE6716F5}" name="Steps" dataDxfId="2"/>
-    <tableColumn id="7" xr3:uid="{2749E69B-C03F-4456-97F1-16E4C7DAB4C8}" name="Test Data" dataDxfId="15"/>
-    <tableColumn id="8" xr3:uid="{10DFC294-FAB0-4D43-8B83-7C0CE4E11BE0}" name="Expected Results" dataDxfId="1"/>
-    <tableColumn id="16" xr3:uid="{2D24DDBD-5A02-4264-B89B-27175D91D43D}" name="Actual result" dataDxfId="14"/>
-    <tableColumn id="9" xr3:uid="{B771E747-8E01-4980-9B14-221C5B00CF89}" name="Post Condition" dataDxfId="13"/>
-    <tableColumn id="10" xr3:uid="{903AF337-308B-4432-90B3-453B150C8696}" name="TC Status" dataDxfId="12"/>
-    <tableColumn id="11" xr3:uid="{DA7982CC-CFB4-46EF-8D7D-498270ACE130}" name="Attachment" dataDxfId="11"/>
-    <tableColumn id="12" xr3:uid="{C3C4BBD3-BE51-4BB4-A9C8-4688454A9D7B}" name="Requirement ID" dataDxfId="10"/>
-    <tableColumn id="13" xr3:uid="{6FFDB195-604A-4141-B2B3-FB2EBCCF9EE1}" name="Type" dataDxfId="9"/>
-    <tableColumn id="14" xr3:uid="{0C076CE8-316D-4323-B69F-E0CA15A82960}" name="Tester" dataDxfId="8"/>
-    <tableColumn id="17" xr3:uid="{C124139E-C07E-4913-834E-C22FF51CDDC5}" name="Execution_Status" dataDxfId="7"/>
-    <tableColumn id="15" xr3:uid="{7B9BAC1F-276D-47AE-B4F7-FBBDF0CA5C1C}" name="Comment" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{6349AC1B-18C1-4513-A98D-74004451BE07}" name="TesTCASE ID" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{316A01E1-D06A-4667-AE3C-453DBC4B1054}" name="Test Cases Title " dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{8F7A3C5E-7DAA-4BE5-BB4C-4242660A0347}" name="valid/invalid" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{6F77ADFD-1C3F-4A08-A6E4-478BE3CD7F59}" name="Environment" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{519F839C-1B74-4449-9BE1-EDCA27C25137}" name="Pre-condition" dataDxfId="14"/>
+    <tableColumn id="6" xr3:uid="{F29F0414-7871-4D01-A1DD-A280EE6716F5}" name="Steps" dataDxfId="13"/>
+    <tableColumn id="7" xr3:uid="{2749E69B-C03F-4456-97F1-16E4C7DAB4C8}" name="Test Data" dataDxfId="12"/>
+    <tableColumn id="8" xr3:uid="{10DFC294-FAB0-4D43-8B83-7C0CE4E11BE0}" name="Expected Results" dataDxfId="11"/>
+    <tableColumn id="16" xr3:uid="{2D24DDBD-5A02-4264-B89B-27175D91D43D}" name="Actual result" dataDxfId="10"/>
+    <tableColumn id="9" xr3:uid="{B771E747-8E01-4980-9B14-221C5B00CF89}" name="Post Condition" dataDxfId="9"/>
+    <tableColumn id="10" xr3:uid="{903AF337-308B-4432-90B3-453B150C8696}" name="TC Status" dataDxfId="8"/>
+    <tableColumn id="11" xr3:uid="{DA7982CC-CFB4-46EF-8D7D-498270ACE130}" name="Attachment" dataDxfId="7"/>
+    <tableColumn id="12" xr3:uid="{C3C4BBD3-BE51-4BB4-A9C8-4688454A9D7B}" name="Requirement ID" dataDxfId="6"/>
+    <tableColumn id="13" xr3:uid="{6FFDB195-604A-4141-B2B3-FB2EBCCF9EE1}" name="Type" dataDxfId="5"/>
+    <tableColumn id="14" xr3:uid="{0C076CE8-316D-4323-B69F-E0CA15A82960}" name="Tester" dataDxfId="4"/>
+    <tableColumn id="17" xr3:uid="{C124139E-C07E-4913-834E-C22FF51CDDC5}" name="Execution_Status" dataDxfId="3"/>
+    <tableColumn id="15" xr3:uid="{7B9BAC1F-276D-47AE-B4F7-FBBDF0CA5C1C}" name="Comment" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="Cart Test Cases-style" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2985,10 +2985,10 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="40" t="s">
+        <v>258</v>
+      </c>
+      <c r="B2" s="38" t="s">
         <v>259</v>
-      </c>
-      <c r="B2" s="38" t="s">
-        <v>260</v>
       </c>
       <c r="C2" s="45" t="s">
         <v>15</v>
@@ -2998,11 +2998,11 @@
       </c>
       <c r="E2" s="54"/>
       <c r="F2" s="41" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G2" s="57"/>
       <c r="H2" s="59" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="I2" s="41"/>
       <c r="J2" s="38" t="s">
@@ -3010,7 +3010,7 @@
       </c>
       <c r="K2" s="38"/>
       <c r="L2" s="38" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="M2" s="38" t="s">
         <v>19</v>
@@ -3022,10 +3022,10 @@
     </row>
     <row r="3" spans="1:15" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A3" s="40" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B3" s="38" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C3" s="45" t="s">
         <v>15</v>
@@ -3035,11 +3035,11 @@
       </c>
       <c r="E3" s="41"/>
       <c r="F3" s="41" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G3" s="57"/>
       <c r="H3" s="38" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="I3" s="41"/>
       <c r="J3" s="38" t="s">
@@ -3047,7 +3047,7 @@
       </c>
       <c r="K3" s="38"/>
       <c r="L3" s="38" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="M3" s="53" t="s">
         <v>21</v>
@@ -3059,10 +3059,10 @@
     </row>
     <row r="4" spans="1:15" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A4" s="40" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B4" s="38" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C4" s="45" t="s">
         <v>15</v>
@@ -3072,11 +3072,11 @@
       </c>
       <c r="E4" s="41"/>
       <c r="F4" s="41" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="G4" s="57"/>
       <c r="H4" s="38" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="I4" s="41"/>
       <c r="J4" s="38" t="s">
@@ -3084,7 +3084,7 @@
       </c>
       <c r="K4" s="38"/>
       <c r="L4" s="38" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="M4" s="53" t="s">
         <v>21</v>
@@ -3096,10 +3096,10 @@
     </row>
     <row r="5" spans="1:15" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A5" s="40" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B5" s="55" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C5" s="45" t="s">
         <v>15</v>
@@ -3109,11 +3109,11 @@
       </c>
       <c r="E5" s="41"/>
       <c r="F5" s="46" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G5" s="57"/>
       <c r="H5" s="53" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="I5" s="41"/>
       <c r="J5" s="38" t="s">
@@ -3121,7 +3121,7 @@
       </c>
       <c r="K5" s="38"/>
       <c r="L5" s="38" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="M5" s="53" t="s">
         <v>21</v>
@@ -3133,10 +3133,10 @@
     </row>
     <row r="6" spans="1:15" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A6" s="40" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B6" s="56" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C6" s="45" t="s">
         <v>15</v>
@@ -3146,11 +3146,11 @@
       </c>
       <c r="E6" s="43"/>
       <c r="F6" s="52" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="G6" s="58"/>
       <c r="H6" s="53" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="I6" s="43"/>
       <c r="J6" s="38" t="s">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="K6" s="39"/>
       <c r="L6" s="38" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="M6" s="53" t="s">
         <v>21</v>
@@ -3170,10 +3170,10 @@
     </row>
     <row r="7" spans="1:15" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A7" s="40" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B7" s="56" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C7" s="45" t="s">
         <v>15</v>
@@ -3183,11 +3183,11 @@
       </c>
       <c r="E7" s="43"/>
       <c r="F7" s="52" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="G7" s="58"/>
       <c r="H7" s="53" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="I7" s="43"/>
       <c r="J7" s="38" t="s">
@@ -3195,7 +3195,7 @@
       </c>
       <c r="K7" s="39"/>
       <c r="L7" s="38" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="M7" s="53" t="s">
         <v>21</v>
@@ -3207,10 +3207,10 @@
     </row>
     <row r="8" spans="1:15" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A8" s="40" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B8" s="56" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C8" s="45" t="s">
         <v>15</v>
@@ -3220,11 +3220,11 @@
       </c>
       <c r="E8" s="43"/>
       <c r="F8" s="52" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="G8" s="58"/>
       <c r="H8" s="53" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="I8" s="43"/>
       <c r="J8" s="38" t="s">
@@ -3232,7 +3232,7 @@
       </c>
       <c r="K8" s="39"/>
       <c r="L8" s="38" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="M8" s="53" t="s">
         <v>21</v>
@@ -3329,10 +3329,10 @@
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="40" t="s">
+        <v>258</v>
+      </c>
+      <c r="B2" s="38" t="s">
         <v>259</v>
-      </c>
-      <c r="B2" s="38" t="s">
-        <v>260</v>
       </c>
       <c r="C2" s="45" t="s">
         <v>15</v>
@@ -3342,16 +3342,16 @@
       </c>
       <c r="E2" s="41"/>
       <c r="F2" s="41" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G2" s="51" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="H2" s="59" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="I2" s="46" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="J2" s="41"/>
       <c r="K2" s="53" t="s">
@@ -3361,7 +3361,7 @@
         <v>18</v>
       </c>
       <c r="M2" s="53" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="N2" s="38" t="s">
         <v>19</v>
@@ -3370,16 +3370,16 @@
         <v>20</v>
       </c>
       <c r="P2" s="50" t="s">
-        <v>258</v>
+        <v>293</v>
       </c>
       <c r="Q2" s="42"/>
     </row>
     <row r="3" spans="1:17" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A3" s="40" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B3" s="38" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C3" s="45" t="s">
         <v>15</v>
@@ -3389,16 +3389,16 @@
       </c>
       <c r="E3" s="41"/>
       <c r="F3" s="41" t="s">
+        <v>264</v>
+      </c>
+      <c r="G3" s="51" t="s">
+        <v>282</v>
+      </c>
+      <c r="H3" s="38" t="s">
         <v>265</v>
       </c>
-      <c r="G3" s="51" t="s">
-        <v>283</v>
-      </c>
-      <c r="H3" s="38" t="s">
-        <v>266</v>
-      </c>
       <c r="I3" s="46" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="J3" s="41"/>
       <c r="K3" s="38" t="s">
@@ -3408,7 +3408,7 @@
         <v>18</v>
       </c>
       <c r="M3" s="53" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="N3" s="53" t="s">
         <v>21</v>
@@ -3417,16 +3417,16 @@
         <v>20</v>
       </c>
       <c r="P3" s="50" t="s">
-        <v>258</v>
+        <v>293</v>
       </c>
       <c r="Q3" s="42"/>
     </row>
     <row r="4" spans="1:17" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A4" s="40" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B4" s="38" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C4" s="45" t="s">
         <v>15</v>
@@ -3436,16 +3436,16 @@
       </c>
       <c r="E4" s="41"/>
       <c r="F4" s="41" t="s">
+        <v>270</v>
+      </c>
+      <c r="G4" s="51" t="s">
+        <v>282</v>
+      </c>
+      <c r="H4" s="38" t="s">
         <v>271</v>
       </c>
-      <c r="G4" s="51" t="s">
-        <v>283</v>
-      </c>
-      <c r="H4" s="38" t="s">
-        <v>272</v>
-      </c>
       <c r="I4" s="46" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="J4" s="41"/>
       <c r="K4" s="38" t="s">
@@ -3455,7 +3455,7 @@
         <v>18</v>
       </c>
       <c r="M4" s="53" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="N4" s="53" t="s">
         <v>21</v>
@@ -3464,16 +3464,16 @@
         <v>20</v>
       </c>
       <c r="P4" s="50" t="s">
-        <v>258</v>
+        <v>293</v>
       </c>
       <c r="Q4" s="42"/>
     </row>
     <row r="5" spans="1:17" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A5" s="40" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B5" s="55" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C5" s="60" t="s">
         <v>23</v>
@@ -3483,16 +3483,16 @@
       </c>
       <c r="E5" s="41"/>
       <c r="F5" s="46" t="s">
+        <v>272</v>
+      </c>
+      <c r="G5" s="51" t="s">
+        <v>282</v>
+      </c>
+      <c r="H5" s="53" t="s">
         <v>273</v>
       </c>
-      <c r="G5" s="51" t="s">
-        <v>283</v>
-      </c>
-      <c r="H5" s="53" t="s">
-        <v>274</v>
-      </c>
       <c r="I5" s="46" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="J5" s="41"/>
       <c r="K5" s="38" t="s">
@@ -3502,7 +3502,7 @@
         <v>18</v>
       </c>
       <c r="M5" s="53" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="N5" s="53" t="s">
         <v>21</v>
@@ -3511,16 +3511,16 @@
         <v>20</v>
       </c>
       <c r="P5" s="50" t="s">
-        <v>258</v>
+        <v>293</v>
       </c>
       <c r="Q5" s="42"/>
     </row>
     <row r="6" spans="1:17" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A6" s="40" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B6" s="56" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C6" s="45" t="s">
         <v>15</v>
@@ -3530,16 +3530,16 @@
       </c>
       <c r="E6" s="41"/>
       <c r="F6" s="52" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="G6" s="51" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="H6" s="53" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="I6" s="46" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="J6" s="41"/>
       <c r="K6" s="38" t="s">
@@ -3549,7 +3549,7 @@
         <v>18</v>
       </c>
       <c r="M6" s="53" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="N6" s="53" t="s">
         <v>21</v>
@@ -3558,16 +3558,16 @@
         <v>20</v>
       </c>
       <c r="P6" s="50" t="s">
-        <v>258</v>
+        <v>293</v>
       </c>
       <c r="Q6" s="42"/>
     </row>
     <row r="7" spans="1:17" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A7" s="40" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B7" s="56" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C7" s="45" t="s">
         <v>15</v>
@@ -3577,16 +3577,16 @@
       </c>
       <c r="E7" s="46"/>
       <c r="F7" s="52" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="G7" s="51" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="H7" s="53" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="I7" s="46" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="J7" s="41"/>
       <c r="K7" s="38" t="s">
@@ -3596,7 +3596,7 @@
         <v>18</v>
       </c>
       <c r="M7" s="53" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="N7" s="53" t="s">
         <v>21</v>
@@ -3605,16 +3605,16 @@
         <v>20</v>
       </c>
       <c r="P7" s="50" t="s">
-        <v>258</v>
+        <v>293</v>
       </c>
       <c r="Q7" s="42"/>
     </row>
     <row r="8" spans="1:17" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A8" s="40" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B8" s="56" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C8" s="45" t="s">
         <v>15</v>
@@ -3624,16 +3624,16 @@
       </c>
       <c r="E8" s="46"/>
       <c r="F8" s="52" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="G8" s="51" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="H8" s="53" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="I8" s="46" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="J8" s="41"/>
       <c r="K8" s="38" t="s">
@@ -3643,7 +3643,7 @@
         <v>18</v>
       </c>
       <c r="M8" s="53" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="N8" s="53" t="s">
         <v>21</v>
@@ -3652,7 +3652,7 @@
         <v>20</v>
       </c>
       <c r="P8" s="50" t="s">
-        <v>258</v>
+        <v>293</v>
       </c>
       <c r="Q8" s="42"/>
     </row>
@@ -3663,10 +3663,10 @@
   </sheetData>
   <phoneticPr fontId="16" type="noConversion"/>
   <conditionalFormatting sqref="P2:P8">
-    <cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="Failed">
+    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Failed">
       <formula>NOT(ISERROR(SEARCH("Failed",P2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="Passed">
+    <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="Passed">
       <formula>NOT(ISERROR(SEARCH("Passed",P2)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>